<commit_message>
Batch status REQUEST_CREATED replaces PENDING
A new batch (and a batch whose carry-forward ran out) has Req_Stat = REQUEST_CREATED.
EXCEPTION_PENDING and the override status PENDING_REVIEW are unchanged. Existing rows need
UPDATE ComplianceRequestControl SET Req_Stat = 'REQUEST_CREATED' WHERE Req_Stat = 'PENDING'.
Glue wheel 0.3.8; docs and the worked-example workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
+++ b/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
@@ -4360,7 +4360,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -4468,7 +4468,7 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K4" s="14" t="n">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K5" s="14" t="n">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K6" s="14" t="n">
@@ -4609,7 +4609,7 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K7" s="14" t="n">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K8" s="14" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K9" s="14" t="n">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K10" s="14" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K11" s="14" t="n">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K12" s="14" t="n">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K13" s="14" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K14" s="14" t="n">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K15" s="14" t="n">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K16" s="14" t="n">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K17" s="14" t="n">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K18" s="14" t="n">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K19" s="14" t="n">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K20" s="14" t="n">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K21" s="14" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K22" s="14" t="n">
@@ -5361,7 +5361,7 @@
       </c>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K23" s="14" t="n">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K24" s="14" t="n">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K25" s="14" t="n">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K26" s="14" t="n">
@@ -5549,7 +5549,7 @@
       </c>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K27" s="14" t="n">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K28" s="14" t="n">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K29" s="14" t="n">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K30" s="14" t="n">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="J31" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K31" s="14" t="n">
@@ -5784,7 +5784,7 @@
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K32" s="14" t="n">
@@ -5831,7 +5831,7 @@
       </c>
       <c r="J33" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K33" s="14" t="n">
@@ -5878,7 +5878,7 @@
       </c>
       <c r="J34" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K34" s="14" t="n">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="J35" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K35" s="14" t="n">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K36" s="14" t="n">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K37" s="14" t="n">
@@ -6066,7 +6066,7 @@
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K38" s="14" t="n">
@@ -6113,7 +6113,7 @@
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K39" s="14" t="n">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K40" s="14" t="n">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K41" s="14" t="n">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K42" s="14" t="n">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K43" s="14" t="n">
@@ -6348,7 +6348,7 @@
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K44" s="14" t="n">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K45" s="14" t="n">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K46" s="14" t="n">
@@ -6489,7 +6489,7 @@
       </c>
       <c r="J47" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K47" s="14" t="n">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K48" s="14" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="J49" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K49" s="14" t="n">
@@ -6630,7 +6630,7 @@
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K50" s="14" t="n">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="J51" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K51" s="14" t="n">
@@ -6724,7 +6724,7 @@
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K52" s="14" t="n">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="J53" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K53" s="14" t="n">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K54" s="14" t="n">
@@ -6865,7 +6865,7 @@
       </c>
       <c r="J55" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K55" s="14" t="n">
@@ -6912,7 +6912,7 @@
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K56" s="14" t="n">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="J57" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K57" s="14" t="n">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="J58" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K58" s="14" t="n">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="J59" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K59" s="14" t="n">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K60" s="14" t="n">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="J61" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K61" s="14" t="n">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="J62" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K62" s="14" t="n">
@@ -7241,7 +7241,7 @@
       </c>
       <c r="J63" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K63" s="14" t="n">
@@ -7288,7 +7288,7 @@
       </c>
       <c r="J64" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K64" s="14" t="n">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="J65" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K65" s="14" t="n">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="J66" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K66" s="14" t="n">
@@ -7429,7 +7429,7 @@
       </c>
       <c r="J67" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K67" s="14" t="n">
@@ -7476,7 +7476,7 @@
       </c>
       <c r="J68" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K68" s="14" t="n">
@@ -7523,7 +7523,7 @@
       </c>
       <c r="J69" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K69" s="14" t="n">
@@ -7570,7 +7570,7 @@
       </c>
       <c r="J70" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K70" s="14" t="n">
@@ -7617,7 +7617,7 @@
       </c>
       <c r="J71" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K71" s="14" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="J72" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K72" s="14" t="n">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="J73" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K73" s="14" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="J74" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K74" s="14" t="n">
@@ -7805,7 +7805,7 @@
       </c>
       <c r="J75" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K75" s="14" t="n">
@@ -7852,7 +7852,7 @@
       </c>
       <c r="J76" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K76" s="14" t="n">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="J77" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K77" s="14" t="n">
@@ -7946,7 +7946,7 @@
       </c>
       <c r="J78" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K78" s="14" t="n">
@@ -7993,7 +7993,7 @@
       </c>
       <c r="J79" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K79" s="14" t="n">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="J80" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K80" s="14" t="n">
@@ -8087,7 +8087,7 @@
       </c>
       <c r="J81" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K81" s="14" t="n">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="J82" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K82" s="14" t="n">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="J83" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K83" s="14" t="n">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="J84" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K84" s="14" t="n">
@@ -8275,7 +8275,7 @@
       </c>
       <c r="J85" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K85" s="14" t="n">
@@ -8322,7 +8322,7 @@
       </c>
       <c r="J86" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K86" s="14" t="n">
@@ -8369,7 +8369,7 @@
       </c>
       <c r="J87" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K87" s="14" t="n">
@@ -8416,7 +8416,7 @@
       </c>
       <c r="J88" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K88" s="14" t="n">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="J89" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K89" s="14" t="n">
@@ -8510,7 +8510,7 @@
       </c>
       <c r="J90" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K90" s="14" t="n">
@@ -8557,7 +8557,7 @@
       </c>
       <c r="J91" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K91" s="14" t="n">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="J92" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K92" s="14" t="n">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="J93" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K93" s="14" t="n">
@@ -8698,7 +8698,7 @@
       </c>
       <c r="J94" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K94" s="14" t="n">
@@ -8745,7 +8745,7 @@
       </c>
       <c r="J95" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K95" s="14" t="n">
@@ -8792,7 +8792,7 @@
       </c>
       <c r="J96" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K96" s="14" t="n">
@@ -8839,7 +8839,7 @@
       </c>
       <c r="J97" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K97" s="14" t="n">
@@ -8886,7 +8886,7 @@
       </c>
       <c r="J98" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K98" s="14" t="n">
@@ -8933,7 +8933,7 @@
       </c>
       <c r="J99" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K99" s="14" t="n">
@@ -8980,7 +8980,7 @@
       </c>
       <c r="J100" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K100" s="14" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="J101" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K101" s="14" t="n">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="J102" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K102" s="14" t="n">
@@ -9121,7 +9121,7 @@
       </c>
       <c r="J103" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K103" s="14" t="n">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J104" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K104" s="14" t="n">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="J105" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K105" s="14" t="n">
@@ -9262,7 +9262,7 @@
       </c>
       <c r="J106" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K106" s="14" t="n">
@@ -9309,7 +9309,7 @@
       </c>
       <c r="J107" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K107" s="14" t="n">
@@ -9356,7 +9356,7 @@
       </c>
       <c r="J108" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K108" s="14" t="n">
@@ -9403,7 +9403,7 @@
       </c>
       <c r="J109" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K109" s="14" t="n">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="J110" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K110" s="14" t="n">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="J111" s="14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>REQUEST_CREATED</t>
         </is>
       </c>
       <c r="K111" s="14" t="n">

</xml_diff>

<commit_message>
Remove email recipients and subject from ComplianceSourceFileConfig
Sucs_Email_Notfn_Id, Failr_Email_Notfn_Id and Email_Subjct_Txt are dropped from the DDL and
the file-config object in both versions; who is notified about a file is handled outside the
framework. NOTIFY no longer reads the file config: it sends every pending event to
DEFAULT_NOTIFY_EMAILS with the subject "[severity] event". Glue wheel 0.3.11; docs and the
example workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
+++ b/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
@@ -2431,7 +2431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2460,6 +2460,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -2528,21 +2529,6 @@
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>Sucs_Email_Notfn_Id</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Failr_Email_Notfn_Id</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr">
-        <is>
-          <t>Email_Subjct_Txt</t>
-        </is>
-      </c>
-      <c r="Q3" s="7" t="inlineStr">
-        <is>
           <t>Active_Ind</t>
         </is>
       </c>
@@ -2607,22 +2593,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N4" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O4" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe ODAG1</t>
-        </is>
-      </c>
-      <c r="Q4" s="8" t="n">
+      <c r="N4" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2686,22 +2657,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O5" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe ODAG1</t>
-        </is>
-      </c>
-      <c r="Q5" s="8" t="n">
+      <c r="N5" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2765,22 +2721,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N6" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O6" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe CDAG1</t>
-        </is>
-      </c>
-      <c r="Q6" s="8" t="n">
+      <c r="N6" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2844,22 +2785,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N7" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O7" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P7" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe SNPCC1</t>
-        </is>
-      </c>
-      <c r="Q7" s="8" t="n">
+      <c r="N7" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2923,22 +2849,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N8" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O8" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P8" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe FA1</t>
-        </is>
-      </c>
-      <c r="Q8" s="8" t="n">
+      <c r="N8" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3002,22 +2913,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N9" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O9" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe FA2</t>
-        </is>
-      </c>
-      <c r="Q9" s="8" t="n">
+      <c r="N9" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3081,22 +2977,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N10" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O10" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe FA3</t>
-        </is>
-      </c>
-      <c r="Q10" s="8" t="n">
+      <c r="N10" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3160,22 +3041,7 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N11" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>universe-team@example.com</t>
-        </is>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>CMS Universe FA4</t>
-        </is>
-      </c>
-      <c r="Q11" s="8" t="n">
+      <c r="N11" s="8" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Y/N indicators, Core_Table_Nm, plain FILE_CHECK columns, source check
- Every yes/no column of the framework's tables is CHAR(1) Y / N instead of SMALLINT 1 / 0
  (Active_Ind, Carry_Fwd_Ind, Src_File_Has_Hdr_Ind, Src_File_Has_Trlr_Ind, Allow_Zero_Rcd_Ind,
  Batch_Close_Ind, Notified_Ind), in the DDL and everywhere the code reads, filters or writes
  them. current_ind of the staging / core data tables is unchanged.
- ComplianceSourceFileConfig.Core_Table_Nm (required) names the core table; it no longer has
  to equal Table_Nm.
- File_Check_Txt (JSON) is replaced by three plain optional columns: File_Rcd_Ty_Txt,
  File_Trlr_Fld_Txt, File_Hdr_Txt (NONE switches a check off for the file).
- FILE_CHECK reports a file whose source is missing from ComplianceSourceSystem or inactive.
- Glue wheel 0.3.12; guides, design note and the example workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
+++ b/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
@@ -733,6 +733,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1602,6 +1603,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1658,8 +1660,10 @@
       <c r="D4" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="E4" s="8" t="n">
-        <v>0</v>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
@@ -1669,8 +1673,10 @@
   AND (EXTRACT(DAY FROM tue) - 1) / 7 + 1 = 3</t>
         </is>
       </c>
-      <c r="G4" s="8" t="n">
-        <v>1</v>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1692,8 +1698,10 @@
       <c r="D5" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="8" t="n">
-        <v>0</v>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -1703,8 +1711,10 @@
   AND (EXTRACT(DAY FROM tue) - 1) / 7 + 1 &lt;&gt; 3</t>
         </is>
       </c>
-      <c r="G5" s="8" t="n">
-        <v>1</v>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1726,12 +1736,16 @@
       <c r="D6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="8" t="n">
-        <v>0</v>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="F6" s="11" t="n"/>
-      <c r="G6" s="8" t="n">
-        <v>1</v>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1769,6 +1783,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1851,8 +1866,10 @@
           <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I4" s="8" t="n">
-        <v>1</v>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1890,8 +1907,10 @@
           <t>SELECT p - 62 AS rpt_start, p - 3 AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I5" s="8" t="n">
-        <v>1</v>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1929,8 +1948,10 @@
           <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I6" s="8" t="n">
-        <v>1</v>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1968,8 +1989,10 @@
           <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I7" s="8" t="n">
-        <v>1</v>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2007,8 +2030,10 @@
           <t>SELECT p - 62 AS rpt_start, p - 3 AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I8" s="8" t="n">
-        <v>1</v>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2046,8 +2071,10 @@
           <t>SELECT p - EXTRACT(DAY FROM p) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I9" s="8" t="n">
-        <v>1</v>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2085,8 +2112,10 @@
           <t>SELECT p - EXTRACT(DAY FROM p) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I10" s="8" t="n">
-        <v>1</v>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -2124,8 +2153,10 @@
           <t>SELECT p - EXTRACT(DAY FROM p) - 13 AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I11" s="8" t="n">
-        <v>1</v>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -2163,8 +2194,10 @@
           <t>SELECT CAST(TRIM(yr) || '-01-01' AS DATE) AS rpt_start, CAST(TRIM(yr) || '-01-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>1</v>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2202,8 +2235,10 @@
           <t>SELECT CAST(TRIM(yr - 1) || '-11-01' AS DATE) AS rpt_start, CAST(TRIM(yr - 1) || '-12-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I13" s="8" t="n">
-        <v>1</v>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2241,8 +2276,10 @@
           <t>SELECT CAST(TRIM(yr - 1) || '-11-01' AS DATE) AS rpt_start, CAST(TRIM(yr) || '-01-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I14" s="8" t="n">
-        <v>1</v>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2280,8 +2317,10 @@
           <t>SELECT CAST(TRIM(yr - 1) || '-11-01' AS DATE) AS rpt_start, CAST(TRIM(yr) || '-01-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I15" s="8" t="n">
-        <v>1</v>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2334,8 +2373,10 @@
           <t>CMS Universe submissions</t>
         </is>
       </c>
-      <c r="C2" s="8" t="n">
-        <v>1</v>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2396,8 +2437,10 @@
           <t>VENDOR</t>
         </is>
       </c>
-      <c r="D2" s="8" t="n">
-        <v>1</v>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -2416,8 +2459,10 @@
           <t>VENDOR</t>
         </is>
       </c>
-      <c r="D3" s="8" t="n">
-        <v>1</v>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2431,7 +2476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2447,7 +2492,7 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="27" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="27" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
@@ -2529,6 +2574,11 @@
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
+          <t>Core_Table_Nm</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
           <t>Active_Ind</t>
         </is>
       </c>
@@ -2564,14 +2614,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0</v>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
@@ -2593,8 +2649,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N4" s="8" t="n">
-        <v>1</v>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>ODAG1</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -2628,14 +2691,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0</v>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
@@ -2657,8 +2726,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N5" s="8" t="n">
-        <v>1</v>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>ODAG1</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2692,14 +2768,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G6" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0</v>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
@@ -2721,8 +2803,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N6" s="8" t="n">
-        <v>1</v>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>CDAG1</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -2756,14 +2845,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0</v>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
@@ -2785,8 +2880,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N7" s="8" t="n">
-        <v>1</v>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>SNPCC1</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2820,14 +2922,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>0</v>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
@@ -2849,8 +2957,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N8" s="8" t="n">
-        <v>1</v>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>FA1</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2884,14 +2999,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G9" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>0</v>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
@@ -2913,8 +3034,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N9" s="8" t="n">
-        <v>1</v>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>FA2</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2948,14 +3076,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>0</v>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
@@ -2977,8 +3111,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N10" s="8" t="n">
-        <v>1</v>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>FA3</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -3012,14 +3153,20 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>0</v>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
@@ -3041,8 +3188,15 @@
           <t>CMS_$ENV_CORE</t>
         </is>
       </c>
-      <c r="N11" s="8" t="n">
-        <v>1</v>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>FA4</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3078,6 +3232,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -4237,6 +4392,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -4337,8 +4493,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K4" s="14" t="n">
-        <v>0</v>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -4384,8 +4542,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K5" s="14" t="n">
-        <v>0</v>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -4431,8 +4591,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K6" s="14" t="n">
-        <v>0</v>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -4478,8 +4640,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K7" s="14" t="n">
-        <v>0</v>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -4525,8 +4689,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K8" s="14" t="n">
-        <v>0</v>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -4572,8 +4738,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K9" s="14" t="n">
-        <v>0</v>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -4619,8 +4787,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K10" s="14" t="n">
-        <v>0</v>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -4666,8 +4836,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K11" s="14" t="n">
-        <v>0</v>
+      <c r="K11" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -4713,8 +4885,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K12" s="14" t="n">
-        <v>0</v>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -4760,8 +4934,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K13" s="14" t="n">
-        <v>0</v>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -4807,8 +4983,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K14" s="14" t="n">
-        <v>0</v>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -4854,8 +5032,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K15" s="14" t="n">
-        <v>0</v>
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -4901,8 +5081,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K16" s="14" t="n">
-        <v>0</v>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -4948,8 +5130,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K17" s="14" t="n">
-        <v>0</v>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -4995,8 +5179,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K18" s="14" t="n">
-        <v>0</v>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -5042,8 +5228,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K19" s="14" t="n">
-        <v>0</v>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -5089,8 +5277,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K20" s="14" t="n">
-        <v>0</v>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -5136,8 +5326,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K21" s="14" t="n">
-        <v>0</v>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -5183,8 +5375,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K22" s="14" t="n">
-        <v>0</v>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -5230,8 +5424,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K23" s="14" t="n">
-        <v>0</v>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -5277,8 +5473,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K24" s="14" t="n">
-        <v>0</v>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -5324,8 +5522,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K25" s="14" t="n">
-        <v>0</v>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -5371,8 +5571,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K26" s="14" t="n">
-        <v>0</v>
+      <c r="K26" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -5418,8 +5620,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K27" s="14" t="n">
-        <v>0</v>
+      <c r="K27" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -5465,8 +5669,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K28" s="14" t="n">
-        <v>0</v>
+      <c r="K28" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -5512,8 +5718,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K29" s="14" t="n">
-        <v>0</v>
+      <c r="K29" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -5559,8 +5767,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K30" s="14" t="n">
-        <v>0</v>
+      <c r="K30" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -5606,8 +5816,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K31" s="14" t="n">
-        <v>0</v>
+      <c r="K31" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -5653,8 +5865,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K32" s="14" t="n">
-        <v>0</v>
+      <c r="K32" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -5700,8 +5914,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K33" s="14" t="n">
-        <v>0</v>
+      <c r="K33" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -5747,8 +5963,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K34" s="14" t="n">
-        <v>0</v>
+      <c r="K34" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -5794,8 +6012,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K35" s="14" t="n">
-        <v>0</v>
+      <c r="K35" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -5841,8 +6061,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K36" s="14" t="n">
-        <v>0</v>
+      <c r="K36" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -5888,8 +6110,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K37" s="14" t="n">
-        <v>0</v>
+      <c r="K37" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -5935,8 +6159,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K38" s="14" t="n">
-        <v>0</v>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -5982,8 +6208,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K39" s="14" t="n">
-        <v>0</v>
+      <c r="K39" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -6029,8 +6257,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K40" s="14" t="n">
-        <v>0</v>
+      <c r="K40" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -6076,8 +6306,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K41" s="14" t="n">
-        <v>0</v>
+      <c r="K41" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -6123,8 +6355,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K42" s="14" t="n">
-        <v>0</v>
+      <c r="K42" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -6170,8 +6404,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K43" s="14" t="n">
-        <v>0</v>
+      <c r="K43" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -6217,8 +6453,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K44" s="14" t="n">
-        <v>0</v>
+      <c r="K44" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -6264,8 +6502,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K45" s="14" t="n">
-        <v>0</v>
+      <c r="K45" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -6311,8 +6551,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K46" s="14" t="n">
-        <v>0</v>
+      <c r="K46" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -6358,8 +6600,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K47" s="14" t="n">
-        <v>0</v>
+      <c r="K47" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -6405,8 +6649,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K48" s="14" t="n">
-        <v>0</v>
+      <c r="K48" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -6452,8 +6698,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K49" s="14" t="n">
-        <v>0</v>
+      <c r="K49" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -6499,8 +6747,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K50" s="14" t="n">
-        <v>0</v>
+      <c r="K50" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -6546,8 +6796,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K51" s="14" t="n">
-        <v>0</v>
+      <c r="K51" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -6593,8 +6845,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K52" s="14" t="n">
-        <v>0</v>
+      <c r="K52" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -6640,8 +6894,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K53" s="14" t="n">
-        <v>0</v>
+      <c r="K53" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -6687,8 +6943,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K54" s="14" t="n">
-        <v>0</v>
+      <c r="K54" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -6734,8 +6992,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K55" s="14" t="n">
-        <v>0</v>
+      <c r="K55" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -6781,8 +7041,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K56" s="14" t="n">
-        <v>0</v>
+      <c r="K56" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -6828,8 +7090,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K57" s="14" t="n">
-        <v>0</v>
+      <c r="K57" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -6875,8 +7139,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K58" s="14" t="n">
-        <v>0</v>
+      <c r="K58" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -6922,8 +7188,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K59" s="14" t="n">
-        <v>0</v>
+      <c r="K59" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -6969,8 +7237,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K60" s="14" t="n">
-        <v>0</v>
+      <c r="K60" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -7016,8 +7286,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K61" s="14" t="n">
-        <v>0</v>
+      <c r="K61" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -7063,8 +7335,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K62" s="14" t="n">
-        <v>0</v>
+      <c r="K62" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -7110,8 +7384,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K63" s="14" t="n">
-        <v>0</v>
+      <c r="K63" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -7157,8 +7433,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K64" s="14" t="n">
-        <v>0</v>
+      <c r="K64" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -7204,8 +7482,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K65" s="14" t="n">
-        <v>0</v>
+      <c r="K65" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -7251,8 +7531,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K66" s="14" t="n">
-        <v>0</v>
+      <c r="K66" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -7298,8 +7580,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K67" s="14" t="n">
-        <v>0</v>
+      <c r="K67" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -7345,8 +7629,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K68" s="14" t="n">
-        <v>0</v>
+      <c r="K68" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -7392,8 +7678,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K69" s="14" t="n">
-        <v>0</v>
+      <c r="K69" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -7439,8 +7727,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K70" s="14" t="n">
-        <v>0</v>
+      <c r="K70" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -7486,8 +7776,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K71" s="14" t="n">
-        <v>0</v>
+      <c r="K71" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -7533,8 +7825,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K72" s="14" t="n">
-        <v>0</v>
+      <c r="K72" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -7580,8 +7874,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K73" s="14" t="n">
-        <v>0</v>
+      <c r="K73" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -7627,8 +7923,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K74" s="14" t="n">
-        <v>0</v>
+      <c r="K74" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -7674,8 +7972,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K75" s="14" t="n">
-        <v>0</v>
+      <c r="K75" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -7721,8 +8021,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K76" s="14" t="n">
-        <v>0</v>
+      <c r="K76" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -7768,8 +8070,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K77" s="14" t="n">
-        <v>0</v>
+      <c r="K77" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -7815,8 +8119,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K78" s="14" t="n">
-        <v>0</v>
+      <c r="K78" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -7862,8 +8168,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K79" s="14" t="n">
-        <v>0</v>
+      <c r="K79" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -7909,8 +8217,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K80" s="14" t="n">
-        <v>0</v>
+      <c r="K80" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -7956,8 +8266,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K81" s="14" t="n">
-        <v>0</v>
+      <c r="K81" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -8003,8 +8315,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K82" s="14" t="n">
-        <v>0</v>
+      <c r="K82" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -8050,8 +8364,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K83" s="14" t="n">
-        <v>0</v>
+      <c r="K83" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -8097,8 +8413,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K84" s="14" t="n">
-        <v>0</v>
+      <c r="K84" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -8144,8 +8462,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K85" s="14" t="n">
-        <v>0</v>
+      <c r="K85" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -8191,8 +8511,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K86" s="14" t="n">
-        <v>0</v>
+      <c r="K86" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -8238,8 +8560,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K87" s="14" t="n">
-        <v>0</v>
+      <c r="K87" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -8285,8 +8609,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K88" s="14" t="n">
-        <v>0</v>
+      <c r="K88" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -8332,8 +8658,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K89" s="14" t="n">
-        <v>0</v>
+      <c r="K89" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -8379,8 +8707,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K90" s="14" t="n">
-        <v>0</v>
+      <c r="K90" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -8426,8 +8756,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K91" s="14" t="n">
-        <v>0</v>
+      <c r="K91" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -8473,8 +8805,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K92" s="14" t="n">
-        <v>0</v>
+      <c r="K92" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -8520,8 +8854,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K93" s="14" t="n">
-        <v>0</v>
+      <c r="K93" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -8567,8 +8903,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K94" s="14" t="n">
-        <v>0</v>
+      <c r="K94" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -8614,8 +8952,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K95" s="14" t="n">
-        <v>0</v>
+      <c r="K95" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -8661,8 +9001,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K96" s="14" t="n">
-        <v>0</v>
+      <c r="K96" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -8708,8 +9050,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K97" s="14" t="n">
-        <v>0</v>
+      <c r="K97" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -8755,8 +9099,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K98" s="14" t="n">
-        <v>0</v>
+      <c r="K98" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -8802,8 +9148,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K99" s="14" t="n">
-        <v>0</v>
+      <c r="K99" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -8849,8 +9197,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K100" s="14" t="n">
-        <v>0</v>
+      <c r="K100" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -8896,8 +9246,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K101" s="14" t="n">
-        <v>0</v>
+      <c r="K101" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -8943,8 +9295,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K102" s="14" t="n">
-        <v>0</v>
+      <c r="K102" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -8990,8 +9344,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K103" s="14" t="n">
-        <v>0</v>
+      <c r="K103" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -9037,8 +9393,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K104" s="14" t="n">
-        <v>0</v>
+      <c r="K104" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -9084,8 +9442,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K105" s="14" t="n">
-        <v>0</v>
+      <c r="K105" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -9131,8 +9491,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K106" s="14" t="n">
-        <v>0</v>
+      <c r="K106" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -9178,8 +9540,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K107" s="14" t="n">
-        <v>0</v>
+      <c r="K107" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -9225,8 +9589,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K108" s="14" t="n">
-        <v>0</v>
+      <c r="K108" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -9272,8 +9638,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K109" s="14" t="n">
-        <v>0</v>
+      <c r="K109" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -9319,8 +9687,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K110" s="14" t="n">
-        <v>0</v>
+      <c r="K110" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -9366,8 +9736,10 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K111" s="14" t="n">
-        <v>0</v>
+      <c r="K111" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Indicators back to SMALLINT 1 / 0
The Y / N form of the yes/no columns (0.3.12) is withdrawn: Active_Ind, Carry_Fwd_Ind,
Src_File_Has_Hdr_Ind, Src_File_Has_Trlr_Ind, Allow_Zero_Rcd_Ind, Batch_Close_Ind and
Notified_Ind are SMALLINT 1 / 0 again in the DDL, the code, the docs and the example workbook.
Core_Table_Nm, the plain FILE_CHECK columns and the source check are kept. Glue wheel 0.3.13.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
+++ b/airflow/compliance_framework/examples/compliance_batch_scenarios.xlsx
@@ -1660,10 +1660,8 @@
       <c r="D4" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="E4" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
@@ -1673,10 +1671,8 @@
   AND (EXTRACT(DAY FROM tue) - 1) / 7 + 1 = 3</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="G4" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1698,10 +1694,8 @@
       <c r="D5" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="E5" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -1711,10 +1705,8 @@
   AND (EXTRACT(DAY FROM tue) - 1) / 7 + 1 &lt;&gt; 3</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="G5" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1736,16 +1728,12 @@
       <c r="D6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="F6" s="11" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="G6" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1866,10 +1854,8 @@
           <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I4" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1907,10 +1893,8 @@
           <t>SELECT p - 62 AS rpt_start, p - 3 AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I5" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1948,10 +1932,8 @@
           <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I6" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1989,10 +1971,8 @@
           <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I7" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -2030,10 +2010,8 @@
           <t>SELECT p - 62 AS rpt_start, p - 3 AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I8" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2071,10 +2049,8 @@
           <t>SELECT p - EXTRACT(DAY FROM p) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I9" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2112,10 +2088,8 @@
           <t>SELECT p - EXTRACT(DAY FROM p) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I10" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2153,10 +2127,8 @@
           <t>SELECT p - EXTRACT(DAY FROM p) - 13 AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I11" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -2194,10 +2166,8 @@
           <t>SELECT CAST(TRIM(yr) || '-01-01' AS DATE) AS rpt_start, CAST(TRIM(yr) || '-01-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I12" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -2235,10 +2205,8 @@
           <t>SELECT CAST(TRIM(yr - 1) || '-11-01' AS DATE) AS rpt_start, CAST(TRIM(yr - 1) || '-12-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I13" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2276,10 +2244,8 @@
           <t>SELECT CAST(TRIM(yr - 1) || '-11-01' AS DATE) AS rpt_start, CAST(TRIM(yr) || '-01-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I14" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2317,10 +2283,8 @@
           <t>SELECT CAST(TRIM(yr - 1) || '-11-01' AS DATE) AS rpt_start, CAST(TRIM(yr) || '-01-31' AS DATE) AS rpt_end FROM (SELECT EXTRACT(YEAR FROM ADD_MONTHS(CAST({period_dt} AS DATE), -1)) AS yr) d</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="I15" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2373,10 +2337,8 @@
           <t>CMS Universe submissions</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="C2" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2437,10 +2399,8 @@
           <t>VENDOR</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="D2" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -2459,10 +2419,8 @@
           <t>VENDOR</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="D3" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2476,7 +2434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2614,20 +2572,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
@@ -2654,10 +2606,8 @@
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="O4" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O4" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -2691,20 +2641,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
@@ -2731,10 +2675,8 @@
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="O5" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O5" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2768,20 +2710,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
@@ -2808,10 +2744,8 @@
           <t>CDAG1</t>
         </is>
       </c>
-      <c r="O6" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O6" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -2845,20 +2779,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
@@ -2885,10 +2813,8 @@
           <t>SNPCC1</t>
         </is>
       </c>
-      <c r="O7" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O7" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -2922,20 +2848,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
@@ -2962,10 +2882,8 @@
           <t>FA1</t>
         </is>
       </c>
-      <c r="O8" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O8" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2999,20 +2917,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
@@ -3039,10 +2951,8 @@
           <t>FA2</t>
         </is>
       </c>
-      <c r="O9" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O9" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3076,20 +2986,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
@@ -3116,10 +3020,8 @@
           <t>FA3</t>
         </is>
       </c>
-      <c r="O10" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O10" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -3153,20 +3055,14 @@
           <t>PIPE</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="G11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
@@ -3193,10 +3089,8 @@
           <t>FA4</t>
         </is>
       </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="O11" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4493,10 +4387,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K4" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4542,10 +4434,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K5" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -4591,10 +4481,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K6" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -4640,10 +4528,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K7" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K7" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4689,10 +4575,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K8" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K8" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4738,10 +4622,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K9" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K9" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -4787,10 +4669,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K10" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K10" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4836,10 +4716,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K11" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K11" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -4885,10 +4763,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K12" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -4934,10 +4810,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K13" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4983,10 +4857,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K14" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -5032,10 +4904,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K15" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K15" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -5081,10 +4951,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K16" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K16" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -5130,10 +4998,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K17" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K17" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -5179,10 +5045,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K18" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K18" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -5228,10 +5092,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K19" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K19" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -5277,10 +5139,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K20" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K20" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -5326,10 +5186,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K21" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K21" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -5375,10 +5233,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K22" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K22" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -5424,10 +5280,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K23" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K23" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -5473,10 +5327,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K24" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -5522,10 +5374,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K25" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -5571,10 +5421,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K26" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K26" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -5620,10 +5468,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K27" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K27" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -5669,10 +5515,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K28" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K28" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -5718,10 +5562,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K29" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K29" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -5767,10 +5609,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K30" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K30" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -5816,10 +5656,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K31" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K31" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -5865,10 +5703,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K32" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K32" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -5914,10 +5750,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K33" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K33" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -5963,10 +5797,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K34" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K34" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -6012,10 +5844,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K35" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K35" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -6061,10 +5891,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K36" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K36" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -6110,10 +5938,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K37" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K37" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -6159,10 +5985,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K38" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K38" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -6208,10 +6032,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K39" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K39" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -6257,10 +6079,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K40" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K40" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -6306,10 +6126,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K41" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K41" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -6355,10 +6173,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K42" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K42" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -6404,10 +6220,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K43" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K43" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -6453,10 +6267,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K44" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K44" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -6502,10 +6314,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K45" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K45" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -6551,10 +6361,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K46" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K46" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -6600,10 +6408,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K47" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K47" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -6649,10 +6455,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K48" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K48" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -6698,10 +6502,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K49" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K49" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -6747,10 +6549,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K50" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K50" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -6796,10 +6596,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K51" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K51" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -6845,10 +6643,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K52" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K52" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -6894,10 +6690,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K53" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K53" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -6943,10 +6737,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K54" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K54" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -6992,10 +6784,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K55" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K55" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -7041,10 +6831,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K56" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K56" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -7090,10 +6878,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K57" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K57" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -7139,10 +6925,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K58" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K58" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -7188,10 +6972,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K59" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K59" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -7237,10 +7019,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K60" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K60" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -7286,10 +7066,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K61" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K61" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -7335,10 +7113,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K62" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K62" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -7384,10 +7160,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K63" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K63" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -7433,10 +7207,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K64" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K64" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -7482,10 +7254,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K65" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K65" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -7531,10 +7301,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K66" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K66" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -7580,10 +7348,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K67" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K67" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -7629,10 +7395,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K68" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K68" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -7678,10 +7442,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K69" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K69" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -7727,10 +7489,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K70" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K70" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -7776,10 +7536,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K71" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K71" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -7825,10 +7583,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K72" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K72" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -7874,10 +7630,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K73" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K73" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -7923,10 +7677,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K74" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K74" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -7972,10 +7724,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K75" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K75" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -8021,10 +7771,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K76" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K76" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -8070,10 +7818,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K77" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K77" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -8119,10 +7865,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K78" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K78" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -8168,10 +7912,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K79" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K79" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -8217,10 +7959,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K80" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K80" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -8266,10 +8006,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K81" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K81" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -8315,10 +8053,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K82" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K82" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -8364,10 +8100,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K83" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K83" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -8413,10 +8147,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K84" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K84" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -8462,10 +8194,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K85" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K85" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -8511,10 +8241,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K86" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K86" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -8560,10 +8288,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K87" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K87" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -8609,10 +8335,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K88" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K88" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -8658,10 +8382,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K89" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K89" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -8707,10 +8429,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K90" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K90" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -8756,10 +8476,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K91" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K91" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -8805,10 +8523,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K92" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K92" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -8854,10 +8570,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K93" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K93" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -8903,10 +8617,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K94" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K94" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -8952,10 +8664,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K95" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K95" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -9001,10 +8711,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K96" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K96" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -9050,10 +8758,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K97" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K97" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -9099,10 +8805,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K98" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K98" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -9148,10 +8852,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K99" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K99" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -9197,10 +8899,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K100" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K100" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -9246,10 +8946,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K101" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K101" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -9295,10 +8993,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K102" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K102" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -9344,10 +9040,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K103" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K103" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -9393,10 +9087,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K104" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K104" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -9442,10 +9134,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K105" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K105" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -9491,10 +9181,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K106" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K106" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -9540,10 +9228,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K107" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K107" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -9589,10 +9275,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K108" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K108" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -9638,10 +9322,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K109" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K109" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -9687,10 +9369,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K110" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K110" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -9736,10 +9416,8 @@
           <t>REQUEST_CREATED</t>
         </is>
       </c>
-      <c r="K111" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+      <c r="K111" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>